<commit_message>
Add Tradeoff Compass v2 and update README and list
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/list.xlsx
+++ b/list.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="10" min="1" max="1"/>
@@ -2145,30 +2145,55 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>AI Creator Ethics — The Tradeoff Compass v2</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>TradeoffCompass.html</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
           <t>AI-Assisted Rubric Creation for Canvas LMS</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>ai-rubric-canvas.html</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>y</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="E78">
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="E79">
         <f>SUM(E2:E76)</f>
         <v/>
       </c>

</xml_diff>